<commit_message>
added video selection algorithm
</commit_message>
<xml_diff>
--- a/smart_product_display_base/Docs/BOM.xlsx
+++ b/smart_product_display_base/Docs/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="46">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -55,6 +55,18 @@
     <t xml:space="preserve">Pin Header 1x20</t>
   </si>
   <si>
+    <t xml:space="preserve">Spacers 8mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">for Holding other end of RPi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spacers 15mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">for Holding PCB</t>
+  </si>
+  <si>
     <t xml:space="preserve">mini-HDMI to HDMI cable</t>
   </si>
   <si>
@@ -64,9 +76,6 @@
     <t xml:space="preserve">Resistors</t>
   </si>
   <si>
-    <t xml:space="preserve">6x1k, 6x330</t>
-  </si>
-  <si>
     <t xml:space="preserve">Capacitor</t>
   </si>
   <si>
@@ -127,7 +136,7 @@
     <t xml:space="preserve">Amazon</t>
   </si>
   <si>
-    <t xml:space="preserve">Power Supply 5v 10Amp</t>
+    <t xml:space="preserve">Power Supply 5v 5Amp</t>
   </si>
   <si>
     <t xml:space="preserve">AC Wire</t>
@@ -508,7 +517,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultColWidth="10.50390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -543,7 +552,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
@@ -551,19 +560,19 @@
         <v>7</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="D2" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="7" t="n">
         <f aca="false">C2*D2</f>
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="9"/>
     </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
@@ -583,8 +592,10 @@
       <c r="F3" s="13"/>
       <c r="G3" s="12"/>
     </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="B4" s="10" t="s">
         <v>9</v>
       </c>
@@ -596,205 +607,203 @@
       <c r="F4" s="13"/>
       <c r="G4" s="12"/>
     </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E5" s="12" t="n">
         <f aca="false">C5*D5</f>
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="F5" s="13"/>
       <c r="G5" s="14"/>
     </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>150</v>
+        <v>3</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" s="12" t="n">
         <f aca="false">C6*D6</f>
-        <v>150</v>
-      </c>
-      <c r="F6" s="13"/>
-      <c r="G6" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="13" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G6" s="14"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E7" s="12" t="n">
         <f aca="false">C7*D7</f>
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F7" s="13" t="s">
         <v>14</v>
       </c>
       <c r="G7" s="14"/>
     </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>5</v>
+        <v>440</v>
       </c>
       <c r="D8" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="12" t="n">
         <f aca="false">C8*D8</f>
-        <v>5</v>
-      </c>
-      <c r="F8" s="13" t="s">
+        <v>440</v>
+      </c>
+      <c r="F8" s="13"/>
+      <c r="G8" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="14"/>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E9" s="12" t="n">
         <f aca="false">C9*D9</f>
+        <v>16</v>
+      </c>
+      <c r="F9" s="13"/>
+      <c r="G9" s="14"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="14"/>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>19</v>
-      </c>
       <c r="C10" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D10" s="11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E10" s="12" t="n">
         <f aca="false">C10*D10</f>
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="F10" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" s="14"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>20</v>
-      </c>
-      <c r="G10" s="14"/>
-    </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>21</v>
       </c>
       <c r="C11" s="11" t="n">
         <v>3</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">C11*D11</f>
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F11" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="14"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="12"/>
-    </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>23</v>
-      </c>
       <c r="C12" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E12" s="12" t="n">
         <f aca="false">C12*D12</f>
-        <v>6</v>
-      </c>
-      <c r="F12" s="13"/>
-      <c r="G12" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="14"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>25</v>
-      </c>
       <c r="C13" s="11" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E13" s="12" t="n">
         <f aca="false">C13*D13</f>
-        <v>36</v>
-      </c>
-      <c r="F13" s="13"/>
-      <c r="G13" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>4</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="12"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>26</v>
@@ -803,205 +812,217 @@
         <v>1</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E14" s="12" t="n">
         <f aca="false">C14*D14</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F14" s="13"/>
       <c r="G14" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E15" s="12" t="n">
         <f aca="false">C15*D15</f>
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="F15" s="13"/>
       <c r="G15" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
+        <v>29</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="E16" s="12" t="n">
         <f aca="false">C16*D16</f>
-        <v>0</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="G16" s="12"/>
-    </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>4</v>
+      </c>
+      <c r="F16" s="13"/>
+      <c r="G16" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
+      <c r="C17" s="11" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="E17" s="12" t="n">
         <f aca="false">C17*D17</f>
-        <v>0</v>
-      </c>
-      <c r="F17" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="13"/>
+      <c r="G17" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G17" s="12"/>
-    </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="11" t="n">
-        <v>75</v>
-      </c>
-      <c r="D18" s="11" t="n">
-        <v>6</v>
-      </c>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
       <c r="E18" s="12" t="n">
         <f aca="false">C18*D18</f>
-        <v>450</v>
-      </c>
-      <c r="F18" s="13"/>
+        <v>0</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="G18" s="12"/>
     </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="11" t="n">
-        <f aca="false">170/2</f>
-        <v>85</v>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>6</v>
-      </c>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
       <c r="E19" s="12" t="n">
         <f aca="false">C19*D19</f>
-        <v>510</v>
-      </c>
-      <c r="F19" s="13"/>
-      <c r="G19" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="F19" s="13" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G19" s="12"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C20" s="11" t="n">
-        <v>390</v>
+        <v>35</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">C20*D20</f>
-        <v>390</v>
+        <v>210</v>
       </c>
       <c r="F20" s="13"/>
-      <c r="G20" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G20" s="12"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>36</v>
       </c>
       <c r="C21" s="11" t="n">
+        <v>120</v>
+      </c>
+      <c r="D21" s="11" t="n">
         <v>6</v>
-      </c>
-      <c r="D21" s="11" t="n">
-        <v>1</v>
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">C21*D21</f>
-        <v>6</v>
+        <v>720</v>
       </c>
       <c r="F21" s="13"/>
-      <c r="G21" s="12"/>
-    </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G21" s="12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C22" s="11" t="n">
-        <v>20</v>
+        <v>230</v>
       </c>
       <c r="D22" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">C22*D22</f>
-        <v>20</v>
+        <v>230</v>
       </c>
       <c r="F22" s="13"/>
-      <c r="G22" s="12"/>
-    </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4"/>
-      <c r="B23" s="10"/>
+      <c r="G22" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="12"/>
+      <c r="D23" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="12" t="n">
+        <f aca="false">C23*D23</f>
+        <v>0</v>
+      </c>
       <c r="F23" s="13"/>
       <c r="G23" s="12"/>
     </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>38</v>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="n">
+        <v>23</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C24" s="11" t="n">
-        <v>300</v>
+        <v>20</v>
       </c>
       <c r="D24" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E24" s="12" t="n">
         <f aca="false">C24*D24</f>
-        <v>300</v>
+        <v>20</v>
       </c>
       <c r="F24" s="13"/>
       <c r="G24" s="12"/>
@@ -1012,50 +1033,79 @@
       <c r="C25" s="11"/>
       <c r="D25" s="11"/>
       <c r="E25" s="12"/>
+      <c r="F25" s="13"/>
       <c r="G25" s="12"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="B26" s="16" t="s">
+      <c r="A26" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C26" s="17" t="n">
-        <v>6000</v>
-      </c>
-      <c r="D26" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="18" t="n">
+      <c r="B26" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="D26" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="12" t="n">
         <f aca="false">C26*D26</f>
-        <v>6000</v>
+        <v>300</v>
       </c>
       <c r="F26" s="13"/>
       <c r="G26" s="12"/>
     </row>
-    <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4"/>
-      <c r="B27" s="19"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="13"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="12"/>
       <c r="G27" s="12"/>
     </row>
-    <row r="28" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1"/>
-      <c r="B28" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="24" t="n">
-        <f aca="false">SUM(E2:E27)</f>
-        <v>10184</v>
-      </c>
-      <c r="F28" s="25"/>
-      <c r="G28" s="21"/>
+    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C28" s="17" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D28" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="18" t="n">
+        <f aca="false">C28*D28</f>
+        <v>6000</v>
+      </c>
+      <c r="F28" s="13"/>
+      <c r="G28" s="12"/>
+    </row>
+    <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1"/>
+      <c r="B30" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="24" t="n">
+        <f aca="false">SUM(E2:E29)</f>
+        <v>10328</v>
+      </c>
+      <c r="F30" s="25"/>
+      <c r="G30" s="21"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
added smoke detector project
</commit_message>
<xml_diff>
--- a/smart_product_display_base/Docs/BOM.xlsx
+++ b/smart_product_display_base/Docs/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -49,7 +49,10 @@
     <t xml:space="preserve">Raspberry Pi Zero W</t>
   </si>
   <si>
-    <t xml:space="preserve">SD Card 64FB</t>
+    <t xml:space="preserve">SD Card 32GB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">imedia</t>
   </si>
   <si>
     <t xml:space="preserve">Pin Header 1x20</t>
@@ -70,7 +73,7 @@
     <t xml:space="preserve">mini-HDMI to HDMI cable</t>
   </si>
   <si>
-    <t xml:space="preserve">imedia store</t>
+    <t xml:space="preserve">amazon</t>
   </si>
   <si>
     <t xml:space="preserve">Resistors</t>
@@ -115,18 +118,6 @@
     <t xml:space="preserve">JST 2P Male</t>
   </si>
   <si>
-    <t xml:space="preserve">Cable 3-wire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">for PIR sensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cable 2-wire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">for LED</t>
-  </si>
-  <si>
     <t xml:space="preserve">PIR proximity sensor</t>
   </si>
   <si>
@@ -143,6 +134,12 @@
   </si>
   <si>
     <t xml:space="preserve">AC Socket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable 8-wires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ethernet cable re-purposed</t>
   </si>
   <si>
     <t xml:space="preserve">**</t>
@@ -517,15 +514,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultColWidth="10.50390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G1048576"/>
+  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="32.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.5"/>
   </cols>
   <sheetData>
@@ -599,20 +596,27 @@
       <c r="B4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="11"/>
+      <c r="C4" s="11" t="n">
+        <v>265</v>
+      </c>
       <c r="D4" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="12"/>
+      <c r="E4" s="12" t="n">
+        <f aca="false">C4*D4</f>
+        <v>265</v>
+      </c>
       <c r="F4" s="13"/>
-      <c r="G4" s="12"/>
+      <c r="G4" s="12" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" s="11" t="n">
         <v>20</v>
@@ -632,7 +636,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="11" t="n">
         <v>3</v>
@@ -645,7 +649,7 @@
         <v>6</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G6" s="14"/>
     </row>
@@ -654,7 +658,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7" s="11" t="n">
         <v>3.5</v>
@@ -667,7 +671,7 @@
         <v>7</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G7" s="14"/>
     </row>
@@ -676,7 +680,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C8" s="11" t="n">
         <v>440</v>
@@ -690,7 +694,7 @@
       </c>
       <c r="F8" s="13"/>
       <c r="G8" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -698,7 +702,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" s="11" t="n">
         <v>1</v>
@@ -718,7 +722,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" s="11" t="n">
         <v>5</v>
@@ -731,7 +735,7 @@
         <v>5</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G10" s="14"/>
     </row>
@@ -740,7 +744,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C11" s="11" t="n">
         <v>3</v>
@@ -753,7 +757,7 @@
         <v>12</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G11" s="14"/>
     </row>
@@ -762,7 +766,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>4</v>
@@ -775,7 +779,7 @@
         <v>16</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G12" s="14"/>
     </row>
@@ -784,7 +788,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C13" s="11" t="n">
         <v>4</v>
@@ -797,7 +801,7 @@
         <v>4</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G13" s="12"/>
     </row>
@@ -806,7 +810,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C14" s="11" t="n">
         <v>1</v>
@@ -820,7 +824,7 @@
       </c>
       <c r="F14" s="13"/>
       <c r="G14" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -828,7 +832,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C15" s="11" t="n">
         <v>6.5</v>
@@ -842,7 +846,7 @@
       </c>
       <c r="F15" s="13"/>
       <c r="G15" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -850,7 +854,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C16" s="11" t="n">
         <v>1</v>
@@ -864,7 +868,7 @@
       </c>
       <c r="F16" s="13"/>
       <c r="G16" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -872,7 +876,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C17" s="11" t="n">
         <v>4.5</v>
@@ -886,227 +890,218 @@
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
+        <v>32</v>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>6</v>
+      </c>
       <c r="E18" s="12" t="n">
         <f aca="false">C18*D18</f>
-        <v>0</v>
-      </c>
-      <c r="F18" s="13" t="s">
-        <v>32</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="F18" s="13"/>
       <c r="G18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
+      <c r="C19" s="11" t="n">
+        <v>120</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>6</v>
+      </c>
       <c r="E19" s="12" t="n">
         <f aca="false">C19*D19</f>
-        <v>0</v>
-      </c>
-      <c r="F19" s="13" t="s">
+        <v>720</v>
+      </c>
+      <c r="F19" s="13"/>
+      <c r="G19" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="G19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C20" s="11" t="n">
-        <v>35</v>
+        <v>230</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">C20*D20</f>
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="F20" s="13"/>
-      <c r="G20" s="12"/>
+      <c r="G20" s="12" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>36</v>
       </c>
       <c r="C21" s="11" t="n">
-        <v>120</v>
+        <v>25</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">C21*D21</f>
-        <v>720</v>
+        <v>25</v>
       </c>
       <c r="F21" s="13"/>
-      <c r="G21" s="12" t="s">
-        <v>37</v>
-      </c>
+      <c r="G21" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C22" s="11" t="n">
-        <v>230</v>
+        <v>20</v>
       </c>
       <c r="D22" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">C22*D22</f>
-        <v>230</v>
+        <v>20</v>
       </c>
       <c r="F22" s="13"/>
-      <c r="G22" s="12" t="s">
-        <v>27</v>
-      </c>
+      <c r="G22" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" s="11"/>
+        <v>38</v>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>36</v>
+      </c>
       <c r="D23" s="11" t="n">
-        <v>1</v>
+        <f aca="false">1.5*4</f>
+        <v>6</v>
       </c>
       <c r="E23" s="12" t="n">
         <f aca="false">C23*D23</f>
-        <v>0</v>
-      </c>
-      <c r="F23" s="13"/>
+        <v>216</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>39</v>
+      </c>
       <c r="G23" s="12"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C24" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="D24" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="12" t="n">
-        <f aca="false">C24*D24</f>
-        <v>20</v>
-      </c>
+    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="12"/>
       <c r="F24" s="13"/>
       <c r="G24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="12"/>
+      <c r="A25" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C25" s="11" t="n">
+        <v>280</v>
+      </c>
+      <c r="D25" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="12" t="n">
+        <f aca="false">C25*D25</f>
+        <v>280</v>
+      </c>
       <c r="F25" s="13"/>
       <c r="G25" s="12"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="10" t="s">
+      <c r="A26" s="4"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="12"/>
+      <c r="G26" s="12"/>
+    </row>
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C26" s="11" t="n">
-        <v>300</v>
-      </c>
-      <c r="D26" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="12" t="n">
-        <f aca="false">C26*D26</f>
-        <v>300</v>
-      </c>
-      <c r="F26" s="13"/>
-      <c r="G26" s="12"/>
-    </row>
-    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="12"/>
+      <c r="B27" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="17" t="n">
+        <v>7500</v>
+      </c>
+      <c r="D27" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="18" t="n">
+        <f aca="false">C27*D27</f>
+        <v>7500</v>
+      </c>
+      <c r="F27" s="13"/>
       <c r="G27" s="12"/>
     </row>
-    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B28" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="C28" s="17" t="n">
-        <v>6000</v>
-      </c>
-      <c r="D28" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="18" t="n">
-        <f aca="false">C28*D28</f>
-        <v>6000</v>
-      </c>
+    <row r="28" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="21"/>
       <c r="F28" s="13"/>
       <c r="G28" s="12"/>
     </row>
     <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4"/>
-      <c r="B29" s="19"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="21"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="12"/>
-    </row>
-    <row r="30" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1"/>
-      <c r="B30" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="C30" s="23"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="24" t="n">
-        <f aca="false">SUM(E2:E29)</f>
-        <v>10328</v>
-      </c>
-      <c r="F30" s="25"/>
-      <c r="G30" s="21"/>
-    </row>
+      <c r="A29" s="1"/>
+      <c r="B29" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="24" t="n">
+        <f aca="false">SUM(E2:E28)</f>
+        <v>12314</v>
+      </c>
+      <c r="F29" s="25"/>
+      <c r="G29" s="21"/>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>